<commit_message>
pics validator: add tracing config; fix missing data in xlsx files; remove carriage return line endings in full.json; re-generate full.json
</commit_message>
<xml_diff>
--- a/data/profiles/mandatory_1547.xlsx
+++ b/data/profiles/mandatory_1547.xlsx
@@ -1,10 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10914"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ande882/projects/ieee-std-1815-2-test-tool/data/profiles/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E7E991CE-03B5-B440-999D-7A8203E805B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView xWindow="240" yWindow="580" windowWidth="16100" windowHeight="9660" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Key" sheetId="1" r:id="rId1"/>
@@ -15,7 +21,7 @@
     <sheet name="CTR" sheetId="6" r:id="rId6"/>
     <sheet name="System Diagrams" sheetId="7" r:id="rId7"/>
   </sheets>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519"/>
 </workbook>
 </file>
 
@@ -4050,8 +4056,8 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -4088,13 +4094,21 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -4132,7 +4146,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -4166,6 +4180,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -4200,9 +4215,10 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -4375,17 +4391,16 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="I2:S50"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="2" spans="9:19">
+    <row r="2" spans="9:19" x14ac:dyDescent="0.2">
       <c r="I2" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="9:19"/>
-    <row r="4" spans="9:19">
+    <row r="4" spans="9:19" x14ac:dyDescent="0.2">
       <c r="I4" t="s">
         <v>1</v>
       </c>
@@ -4408,12 +4423,12 @@
         <v>7</v>
       </c>
     </row>
-    <row r="5" spans="9:19">
+    <row r="5" spans="9:19" x14ac:dyDescent="0.2">
       <c r="I5" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="6" spans="9:19">
+    <row r="6" spans="9:19" x14ac:dyDescent="0.2">
       <c r="I6" t="s">
         <v>9</v>
       </c>
@@ -4436,7 +4451,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="9:19">
+    <row r="7" spans="9:19" x14ac:dyDescent="0.2">
       <c r="I7" t="s">
         <v>10</v>
       </c>
@@ -4462,7 +4477,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="8" spans="9:19">
+    <row r="8" spans="9:19" x14ac:dyDescent="0.2">
       <c r="I8" t="s">
         <v>12</v>
       </c>
@@ -4491,7 +4506,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="9" spans="9:19">
+    <row r="9" spans="9:19" x14ac:dyDescent="0.2">
       <c r="I9" t="s">
         <v>15</v>
       </c>
@@ -4514,7 +4529,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="9:19">
+    <row r="10" spans="9:19" x14ac:dyDescent="0.2">
       <c r="I10" t="s">
         <v>16</v>
       </c>
@@ -4537,7 +4552,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="9:19">
+    <row r="11" spans="9:19" x14ac:dyDescent="0.2">
       <c r="I11" t="s">
         <v>17</v>
       </c>
@@ -4560,13 +4575,12 @@
         <v>586</v>
       </c>
     </row>
-    <row r="12" spans="9:19"/>
-    <row r="13" spans="9:19">
+    <row r="13" spans="9:19" x14ac:dyDescent="0.2">
       <c r="I13" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="14" spans="9:19">
+    <row r="14" spans="9:19" x14ac:dyDescent="0.2">
       <c r="I14" t="s">
         <v>21</v>
       </c>
@@ -4592,7 +4606,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="15" spans="9:19">
+    <row r="15" spans="9:19" x14ac:dyDescent="0.2">
       <c r="I15" t="s">
         <v>24</v>
       </c>
@@ -4609,7 +4623,7 @@
         <v>2300</v>
       </c>
     </row>
-    <row r="16" spans="9:19">
+    <row r="16" spans="9:19" x14ac:dyDescent="0.2">
       <c r="I16" t="s">
         <v>26</v>
       </c>
@@ -4632,7 +4646,7 @@
         <v>3000</v>
       </c>
     </row>
-    <row r="17" spans="9:19">
+    <row r="17" spans="9:19" x14ac:dyDescent="0.2">
       <c r="I17" t="s">
         <v>28</v>
       </c>
@@ -4655,7 +4669,7 @@
         <v>3500</v>
       </c>
     </row>
-    <row r="18" spans="9:19">
+    <row r="18" spans="9:19" x14ac:dyDescent="0.2">
       <c r="I18" t="s">
         <v>30</v>
       </c>
@@ -4666,8 +4680,7 @@
         <v>4000</v>
       </c>
     </row>
-    <row r="19" spans="9:19"/>
-    <row r="20" spans="9:19">
+    <row r="20" spans="9:19" x14ac:dyDescent="0.2">
       <c r="I20" t="s">
         <v>31</v>
       </c>
@@ -4690,7 +4703,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="21" spans="9:19">
+    <row r="21" spans="9:19" x14ac:dyDescent="0.2">
       <c r="I21" t="s">
         <v>33</v>
       </c>
@@ -4722,7 +4735,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="22" spans="9:19">
+    <row r="22" spans="9:19" x14ac:dyDescent="0.2">
       <c r="J22" t="s">
         <v>36</v>
       </c>
@@ -4742,7 +4755,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="23" spans="9:19">
+    <row r="23" spans="9:19" x14ac:dyDescent="0.2">
       <c r="J23" t="s">
         <v>37</v>
       </c>
@@ -4762,7 +4775,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="24" spans="9:19">
+    <row r="24" spans="9:19" x14ac:dyDescent="0.2">
       <c r="I24" t="s">
         <v>38</v>
       </c>
@@ -4791,7 +4804,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="25" spans="9:19">
+    <row r="25" spans="9:19" x14ac:dyDescent="0.2">
       <c r="J25" t="s">
         <v>41</v>
       </c>
@@ -4811,7 +4824,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="9:19">
+    <row r="26" spans="9:19" x14ac:dyDescent="0.2">
       <c r="J26" t="s">
         <v>42</v>
       </c>
@@ -4828,7 +4841,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="27" spans="9:19">
+    <row r="27" spans="9:19" x14ac:dyDescent="0.2">
       <c r="I27" t="s">
         <v>43</v>
       </c>
@@ -4857,7 +4870,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="28" spans="9:19">
+    <row r="28" spans="9:19" x14ac:dyDescent="0.2">
       <c r="J28" t="s">
         <v>46</v>
       </c>
@@ -4877,7 +4890,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="9:19">
+    <row r="29" spans="9:19" x14ac:dyDescent="0.2">
       <c r="J29" t="s">
         <v>47</v>
       </c>
@@ -4894,7 +4907,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="30" spans="9:19">
+    <row r="30" spans="9:19" x14ac:dyDescent="0.2">
       <c r="I30" t="s">
         <v>48</v>
       </c>
@@ -4923,7 +4936,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="31" spans="9:19">
+    <row r="31" spans="9:19" x14ac:dyDescent="0.2">
       <c r="J31" t="s">
         <v>51</v>
       </c>
@@ -4946,7 +4959,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="32" spans="9:19">
+    <row r="32" spans="9:19" x14ac:dyDescent="0.2">
       <c r="J32" t="s">
         <v>53</v>
       </c>
@@ -4963,7 +4976,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="33" spans="9:19">
+    <row r="33" spans="9:19" x14ac:dyDescent="0.2">
       <c r="I33" t="s">
         <v>54</v>
       </c>
@@ -4974,7 +4987,7 @@
         <v>30000</v>
       </c>
     </row>
-    <row r="34" spans="9:19">
+    <row r="34" spans="9:19" x14ac:dyDescent="0.2">
       <c r="I34" t="s">
         <v>56</v>
       </c>
@@ -4997,7 +5010,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="35" spans="9:19">
+    <row r="35" spans="9:19" x14ac:dyDescent="0.2">
       <c r="I35" t="s">
         <v>58</v>
       </c>
@@ -5017,7 +5030,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="36" spans="9:19">
+    <row r="36" spans="9:19" x14ac:dyDescent="0.2">
       <c r="I36" t="s">
         <v>62</v>
       </c>
@@ -5025,8 +5038,7 @@
         <v>65535</v>
       </c>
     </row>
-    <row r="37" spans="9:19"/>
-    <row r="38" spans="9:19">
+    <row r="38" spans="9:19" x14ac:dyDescent="0.2">
       <c r="I38" t="s">
         <v>63</v>
       </c>
@@ -5037,7 +5049,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="39" spans="9:19">
+    <row r="39" spans="9:19" x14ac:dyDescent="0.2">
       <c r="I39" t="s">
         <v>66</v>
       </c>
@@ -5048,7 +5060,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="40" spans="9:19">
+    <row r="40" spans="9:19" x14ac:dyDescent="0.2">
       <c r="I40" t="s">
         <v>69</v>
       </c>
@@ -5059,7 +5071,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="41" spans="9:19">
+    <row r="41" spans="9:19" x14ac:dyDescent="0.2">
       <c r="I41" t="s">
         <v>72</v>
       </c>
@@ -5070,8 +5082,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="42" spans="9:19"/>
-    <row r="43" spans="9:19">
+    <row r="43" spans="9:19" x14ac:dyDescent="0.2">
       <c r="I43" t="s">
         <v>75</v>
       </c>
@@ -5082,7 +5093,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="44" spans="9:19">
+    <row r="44" spans="9:19" x14ac:dyDescent="0.2">
       <c r="I44" t="s">
         <v>77</v>
       </c>
@@ -5093,7 +5104,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="45" spans="9:19">
+    <row r="45" spans="9:19" x14ac:dyDescent="0.2">
       <c r="I45" t="s">
         <v>79</v>
       </c>
@@ -5104,7 +5115,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="46" spans="9:19">
+    <row r="46" spans="9:19" x14ac:dyDescent="0.2">
       <c r="I46" t="s">
         <v>81</v>
       </c>
@@ -5115,8 +5126,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="47" spans="9:19"/>
-    <row r="48" spans="9:19">
+    <row r="48" spans="9:19" x14ac:dyDescent="0.2">
       <c r="I48" t="s">
         <v>83</v>
       </c>
@@ -5127,7 +5137,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="49" spans="9:13">
+    <row r="49" spans="9:13" x14ac:dyDescent="0.2">
       <c r="I49" t="s">
         <v>85</v>
       </c>
@@ -5138,7 +5148,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="50" spans="9:13">
+    <row r="50" spans="9:13" x14ac:dyDescent="0.2">
       <c r="I50" t="s">
         <v>87</v>
       </c>
@@ -5155,11 +5165,11 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:J9"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:10">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>89</v>
       </c>
@@ -5182,7 +5192,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="2" spans="1:10">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
       <c r="E2" t="s">
         <v>96</v>
       </c>
@@ -5202,7 +5212,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="3" spans="1:10">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>102</v>
       </c>
@@ -5231,7 +5241,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="4" spans="1:10">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>110</v>
       </c>
@@ -5260,7 +5270,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="5" spans="1:10">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>118</v>
       </c>
@@ -5289,7 +5299,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="6" spans="1:10">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>123</v>
       </c>
@@ -5318,7 +5328,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="7" spans="1:10">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>128</v>
       </c>
@@ -5347,7 +5357,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="8" spans="1:10">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>133</v>
       </c>
@@ -5376,7 +5386,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="9" spans="1:10">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>138</v>
       </c>
@@ -5411,11 +5421,11 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:K127"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:11">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>142</v>
       </c>
@@ -5441,7 +5451,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="2" spans="1:11">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
       <c r="F2" t="s">
         <v>96</v>
       </c>
@@ -5461,7 +5471,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="3" spans="1:11">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>145</v>
       </c>
@@ -5490,7 +5500,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="4" spans="1:11">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>151</v>
       </c>
@@ -5519,7 +5529,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="5" spans="1:11">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>156</v>
       </c>
@@ -5548,7 +5558,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="6" spans="1:11">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>162</v>
       </c>
@@ -5577,7 +5587,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="7" spans="1:11">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>166</v>
       </c>
@@ -5606,7 +5616,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="8" spans="1:11">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>172</v>
       </c>
@@ -5635,7 +5645,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="9" spans="1:11">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>176</v>
       </c>
@@ -5664,7 +5674,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="10" spans="1:11">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>180</v>
       </c>
@@ -5693,7 +5703,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="11" spans="1:11">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>183</v>
       </c>
@@ -5722,7 +5732,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="12" spans="1:11">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>186</v>
       </c>
@@ -5751,7 +5761,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="13" spans="1:11">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>189</v>
       </c>
@@ -5780,7 +5790,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="14" spans="1:11">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>192</v>
       </c>
@@ -5809,7 +5819,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="15" spans="1:11">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>195</v>
       </c>
@@ -5838,7 +5848,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="16" spans="1:11">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>115</v>
       </c>
@@ -5870,7 +5880,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="17" spans="1:10">
+    <row r="17" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>121</v>
       </c>
@@ -5902,7 +5912,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="18" spans="1:10">
+    <row r="18" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>126</v>
       </c>
@@ -5934,7 +5944,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="19" spans="1:10">
+    <row r="19" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>131</v>
       </c>
@@ -5966,7 +5976,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="20" spans="1:10">
+    <row r="20" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>136</v>
       </c>
@@ -5998,7 +6008,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="21" spans="1:10">
+    <row r="21" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>206</v>
       </c>
@@ -6030,7 +6040,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="22" spans="1:10">
+    <row r="22" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>210</v>
       </c>
@@ -6053,7 +6063,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="23" spans="1:10">
+    <row r="23" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>214</v>
       </c>
@@ -6076,7 +6086,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="24" spans="1:10">
+    <row r="24" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>216</v>
       </c>
@@ -6099,7 +6109,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="25" spans="1:10">
+    <row r="25" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>219</v>
       </c>
@@ -6122,7 +6132,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="26" spans="1:10">
+    <row r="26" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>221</v>
       </c>
@@ -6145,7 +6155,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="27" spans="1:10">
+    <row r="27" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>224</v>
       </c>
@@ -6168,7 +6178,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="28" spans="1:10">
+    <row r="28" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>226</v>
       </c>
@@ -6191,7 +6201,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="29" spans="1:10">
+    <row r="29" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>229</v>
       </c>
@@ -6214,7 +6224,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="30" spans="1:10">
+    <row r="30" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>231</v>
       </c>
@@ -6237,7 +6247,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="31" spans="1:10">
+    <row r="31" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
         <v>234</v>
       </c>
@@ -6260,7 +6270,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="32" spans="1:10">
+    <row r="32" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
         <v>236</v>
       </c>
@@ -6283,7 +6293,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="33" spans="1:8">
+    <row r="33" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
         <v>239</v>
       </c>
@@ -6306,7 +6316,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="34" spans="1:8">
+    <row r="34" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
         <v>241</v>
       </c>
@@ -6329,7 +6339,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="35" spans="1:8">
+    <row r="35" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
         <v>246</v>
       </c>
@@ -6352,7 +6362,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="36" spans="1:8">
+    <row r="36" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
         <v>251</v>
       </c>
@@ -6375,7 +6385,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="37" spans="1:8">
+    <row r="37" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
         <v>254</v>
       </c>
@@ -6398,7 +6408,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="38" spans="1:8">
+    <row r="38" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
         <v>259</v>
       </c>
@@ -6421,7 +6431,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="39" spans="1:8">
+    <row r="39" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
         <v>264</v>
       </c>
@@ -6444,7 +6454,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="40" spans="1:8">
+    <row r="40" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
         <v>267</v>
       </c>
@@ -6467,7 +6477,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="41" spans="1:8">
+    <row r="41" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
         <v>269</v>
       </c>
@@ -6490,7 +6500,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="42" spans="1:8">
+    <row r="42" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
         <v>272</v>
       </c>
@@ -6513,7 +6523,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="43" spans="1:8">
+    <row r="43" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
         <v>274</v>
       </c>
@@ -6536,7 +6546,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="44" spans="1:8">
+    <row r="44" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
         <v>277</v>
       </c>
@@ -6559,7 +6569,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="45" spans="1:8">
+    <row r="45" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
         <v>279</v>
       </c>
@@ -6582,7 +6592,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="46" spans="1:8">
+    <row r="46" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
         <v>282</v>
       </c>
@@ -6605,7 +6615,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="47" spans="1:8">
+    <row r="47" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
         <v>284</v>
       </c>
@@ -6628,7 +6638,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="48" spans="1:8">
+    <row r="48" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
         <v>287</v>
       </c>
@@ -6651,7 +6661,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="49" spans="1:8">
+    <row r="49" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
         <v>289</v>
       </c>
@@ -6674,7 +6684,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="50" spans="1:8">
+    <row r="50" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
         <v>292</v>
       </c>
@@ -6697,7 +6707,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="51" spans="1:8">
+    <row r="51" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
         <v>294</v>
       </c>
@@ -6720,7 +6730,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="52" spans="1:8">
+    <row r="52" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
         <v>299</v>
       </c>
@@ -6743,7 +6753,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="53" spans="1:8">
+    <row r="53" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
         <v>302</v>
       </c>
@@ -6766,7 +6776,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="54" spans="1:8">
+    <row r="54" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
         <v>305</v>
       </c>
@@ -6789,7 +6799,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="55" spans="1:8">
+    <row r="55" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
         <v>308</v>
       </c>
@@ -6812,7 +6822,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="56" spans="1:8">
+    <row r="56" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
         <v>311</v>
       </c>
@@ -6835,7 +6845,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="57" spans="1:8">
+    <row r="57" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
         <v>313</v>
       </c>
@@ -6858,7 +6868,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="58" spans="1:8">
+    <row r="58" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
         <v>315</v>
       </c>
@@ -6881,7 +6891,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="59" spans="1:8">
+    <row r="59" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
         <v>318</v>
       </c>
@@ -6904,7 +6914,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="60" spans="1:8">
+    <row r="60" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
         <v>321</v>
       </c>
@@ -6927,7 +6937,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="61" spans="1:8">
+    <row r="61" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
         <v>325</v>
       </c>
@@ -6950,7 +6960,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="62" spans="1:8">
+    <row r="62" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
         <v>328</v>
       </c>
@@ -6973,7 +6983,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="63" spans="1:8">
+    <row r="63" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
         <v>331</v>
       </c>
@@ -6996,7 +7006,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="64" spans="1:8">
+    <row r="64" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
         <v>334</v>
       </c>
@@ -7019,7 +7029,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="65" spans="1:8">
+    <row r="65" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A65" t="s">
         <v>336</v>
       </c>
@@ -7042,7 +7052,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="66" spans="1:8">
+    <row r="66" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A66" t="s">
         <v>338</v>
       </c>
@@ -7065,7 +7075,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="67" spans="1:8">
+    <row r="67" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A67" t="s">
         <v>340</v>
       </c>
@@ -7088,7 +7098,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="68" spans="1:8">
+    <row r="68" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A68" t="s">
         <v>343</v>
       </c>
@@ -7111,7 +7121,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="69" spans="1:8">
+    <row r="69" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A69" t="s">
         <v>345</v>
       </c>
@@ -7134,7 +7144,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="70" spans="1:8">
+    <row r="70" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A70" t="s">
         <v>348</v>
       </c>
@@ -7157,7 +7167,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="71" spans="1:8">
+    <row r="71" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A71" t="s">
         <v>351</v>
       </c>
@@ -7180,7 +7190,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="72" spans="1:8">
+    <row r="72" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A72" t="s">
         <v>354</v>
       </c>
@@ -7203,7 +7213,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="73" spans="1:8">
+    <row r="73" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A73" t="s">
         <v>357</v>
       </c>
@@ -7226,7 +7236,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="74" spans="1:8">
+    <row r="74" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A74" t="s">
         <v>360</v>
       </c>
@@ -7249,7 +7259,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="75" spans="1:8">
+    <row r="75" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A75" t="s">
         <v>365</v>
       </c>
@@ -7272,7 +7282,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="76" spans="1:8">
+    <row r="76" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A76" t="s">
         <v>368</v>
       </c>
@@ -7295,7 +7305,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="77" spans="1:8">
+    <row r="77" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A77" t="s">
         <v>373</v>
       </c>
@@ -7318,7 +7328,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="78" spans="1:8">
+    <row r="78" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A78" t="s">
         <v>378</v>
       </c>
@@ -7341,7 +7351,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="79" spans="1:8">
+    <row r="79" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A79" t="s">
         <v>383</v>
       </c>
@@ -7364,7 +7374,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="80" spans="1:8">
+    <row r="80" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A80" t="s">
         <v>388</v>
       </c>
@@ -7387,7 +7397,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="81" spans="1:8">
+    <row r="81" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A81" t="s">
         <v>391</v>
       </c>
@@ -7410,7 +7420,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="82" spans="1:8">
+    <row r="82" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A82" t="s">
         <v>394</v>
       </c>
@@ -7433,7 +7443,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="83" spans="1:8">
+    <row r="83" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A83" t="s">
         <v>397</v>
       </c>
@@ -7456,7 +7466,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="84" spans="1:8">
+    <row r="84" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A84" t="s">
         <v>400</v>
       </c>
@@ -7479,7 +7489,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="85" spans="1:8">
+    <row r="85" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A85" t="s">
         <v>403</v>
       </c>
@@ -7502,7 +7512,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="86" spans="1:8">
+    <row r="86" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A86" t="s">
         <v>406</v>
       </c>
@@ -7525,7 +7535,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="87" spans="1:8">
+    <row r="87" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A87" t="s">
         <v>409</v>
       </c>
@@ -7548,7 +7558,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="88" spans="1:8">
+    <row r="88" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A88" t="s">
         <v>412</v>
       </c>
@@ -7571,7 +7581,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="89" spans="1:8">
+    <row r="89" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A89" t="s">
         <v>415</v>
       </c>
@@ -7594,7 +7604,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="90" spans="1:8">
+    <row r="90" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A90" t="s">
         <v>418</v>
       </c>
@@ -7617,7 +7627,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="91" spans="1:8">
+    <row r="91" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A91" t="s">
         <v>421</v>
       </c>
@@ -7640,7 +7650,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="92" spans="1:8">
+    <row r="92" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A92" t="s">
         <v>424</v>
       </c>
@@ -7663,7 +7673,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="93" spans="1:8">
+    <row r="93" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A93" t="s">
         <v>427</v>
       </c>
@@ -7686,7 +7696,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="94" spans="1:8">
+    <row r="94" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A94" t="s">
         <v>430</v>
       </c>
@@ -7709,7 +7719,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="95" spans="1:8">
+    <row r="95" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A95" t="s">
         <v>433</v>
       </c>
@@ -7732,7 +7742,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="96" spans="1:8">
+    <row r="96" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A96" t="s">
         <v>436</v>
       </c>
@@ -7755,7 +7765,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="97" spans="1:8">
+    <row r="97" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A97" t="s">
         <v>438</v>
       </c>
@@ -7778,7 +7788,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="98" spans="1:8">
+    <row r="98" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A98" t="s">
         <v>440</v>
       </c>
@@ -7801,7 +7811,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="99" spans="1:8">
+    <row r="99" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A99" t="s">
         <v>443</v>
       </c>
@@ -7824,7 +7834,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="100" spans="1:8">
+    <row r="100" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A100" t="s">
         <v>446</v>
       </c>
@@ -7847,7 +7857,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="101" spans="1:8">
+    <row r="101" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A101" t="s">
         <v>449</v>
       </c>
@@ -7870,7 +7880,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="102" spans="1:8">
+    <row r="102" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A102" t="s">
         <v>452</v>
       </c>
@@ -7893,7 +7903,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="103" spans="1:8">
+    <row r="103" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A103" t="s">
         <v>455</v>
       </c>
@@ -7916,7 +7926,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="104" spans="1:8">
+    <row r="104" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A104" t="s">
         <v>458</v>
       </c>
@@ -7939,7 +7949,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="105" spans="1:8">
+    <row r="105" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A105" t="s">
         <v>461</v>
       </c>
@@ -7962,7 +7972,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="106" spans="1:8">
+    <row r="106" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A106" t="s">
         <v>464</v>
       </c>
@@ -7985,7 +7995,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="107" spans="1:8">
+    <row r="107" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A107" t="s">
         <v>467</v>
       </c>
@@ -8008,7 +8018,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="108" spans="1:8">
+    <row r="108" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A108" t="s">
         <v>470</v>
       </c>
@@ -8031,7 +8041,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="109" spans="1:8">
+    <row r="109" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A109" t="s">
         <v>473</v>
       </c>
@@ -8054,7 +8064,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="110" spans="1:8">
+    <row r="110" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A110" t="s">
         <v>476</v>
       </c>
@@ -8077,7 +8087,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="111" spans="1:8">
+    <row r="111" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A111" t="s">
         <v>479</v>
       </c>
@@ -8100,7 +8110,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="112" spans="1:8">
+    <row r="112" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A112" t="s">
         <v>482</v>
       </c>
@@ -8123,7 +8133,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="113" spans="1:8">
+    <row r="113" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A113" t="s">
         <v>485</v>
       </c>
@@ -8146,7 +8156,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="114" spans="1:8">
+    <row r="114" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A114" t="s">
         <v>488</v>
       </c>
@@ -8169,7 +8179,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="115" spans="1:8">
+    <row r="115" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A115" t="s">
         <v>491</v>
       </c>
@@ -8192,7 +8202,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="116" spans="1:8">
+    <row r="116" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A116" t="s">
         <v>494</v>
       </c>
@@ -8215,7 +8225,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="117" spans="1:8">
+    <row r="117" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A117" t="s">
         <v>497</v>
       </c>
@@ -8238,7 +8248,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="118" spans="1:8">
+    <row r="118" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A118" t="s">
         <v>500</v>
       </c>
@@ -8261,7 +8271,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="119" spans="1:8">
+    <row r="119" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A119" t="s">
         <v>503</v>
       </c>
@@ -8284,7 +8294,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="120" spans="1:8">
+    <row r="120" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A120" t="s">
         <v>506</v>
       </c>
@@ -8307,7 +8317,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="121" spans="1:8">
+    <row r="121" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A121" t="s">
         <v>509</v>
       </c>
@@ -8330,7 +8340,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="122" spans="1:8">
+    <row r="122" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A122" t="s">
         <v>512</v>
       </c>
@@ -8353,7 +8363,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="123" spans="1:8">
+    <row r="123" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A123" t="s">
         <v>515</v>
       </c>
@@ -8376,7 +8386,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="124" spans="1:8">
+    <row r="124" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A124" t="s">
         <v>518</v>
       </c>
@@ -8399,7 +8409,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="125" spans="1:8">
+    <row r="125" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A125" t="s">
         <v>521</v>
       </c>
@@ -8422,7 +8432,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="126" spans="1:8">
+    <row r="126" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A126" t="s">
         <v>524</v>
       </c>
@@ -8445,7 +8455,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="127" spans="1:8">
+    <row r="127" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A127" t="s">
         <v>527</v>
       </c>
@@ -8474,11 +8484,11 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:O72"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:15">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>89</v>
       </c>
@@ -8504,7 +8514,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="2" spans="1:15">
+    <row r="2" spans="1:15" x14ac:dyDescent="0.2">
       <c r="C2" t="s">
         <v>533</v>
       </c>
@@ -8542,7 +8552,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="3" spans="1:15">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>541</v>
       </c>
@@ -8580,7 +8590,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="4" spans="1:15">
+    <row r="4" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>547</v>
       </c>
@@ -8618,7 +8628,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="5" spans="1:15">
+    <row r="5" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>551</v>
       </c>
@@ -8656,7 +8666,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="6" spans="1:15">
+    <row r="6" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>555</v>
       </c>
@@ -8694,7 +8704,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="7" spans="1:15">
+    <row r="7" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>559</v>
       </c>
@@ -8732,7 +8742,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="8" spans="1:15">
+    <row r="8" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>563</v>
       </c>
@@ -8770,7 +8780,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="9" spans="1:15">
+    <row r="9" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>567</v>
       </c>
@@ -8784,7 +8794,7 @@
         <v>70000</v>
       </c>
       <c r="E9">
-        <v>0.001</v>
+        <v>1E-3</v>
       </c>
       <c r="F9">
         <v>0</v>
@@ -8808,7 +8818,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="10" spans="1:15">
+    <row r="10" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>572</v>
       </c>
@@ -8822,7 +8832,7 @@
         <v>2147483647</v>
       </c>
       <c r="E10">
-        <v>0.001</v>
+        <v>1E-3</v>
       </c>
       <c r="F10">
         <v>0</v>
@@ -8846,7 +8856,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="11" spans="1:15">
+    <row r="11" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>578</v>
       </c>
@@ -8860,7 +8870,7 @@
         <v>0</v>
       </c>
       <c r="E11">
-        <v>0.001</v>
+        <v>1E-3</v>
       </c>
       <c r="F11">
         <v>0</v>
@@ -8884,7 +8894,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="12" spans="1:15">
+    <row r="12" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>582</v>
       </c>
@@ -8898,7 +8908,7 @@
         <v>2147483647</v>
       </c>
       <c r="E12">
-        <v>0.001</v>
+        <v>1E-3</v>
       </c>
       <c r="F12">
         <v>0</v>
@@ -8922,7 +8932,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="13" spans="1:15">
+    <row r="13" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>587</v>
       </c>
@@ -8957,7 +8967,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="14" spans="1:15">
+    <row r="14" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>592</v>
       </c>
@@ -8992,7 +9002,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="15" spans="1:15">
+    <row r="15" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>596</v>
       </c>
@@ -9030,7 +9040,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="16" spans="1:15">
+    <row r="16" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>602</v>
       </c>
@@ -9068,7 +9078,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="17" spans="1:12">
+    <row r="17" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>607</v>
       </c>
@@ -9106,7 +9116,7 @@
         <v>612</v>
       </c>
     </row>
-    <row r="18" spans="1:12">
+    <row r="18" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>613</v>
       </c>
@@ -9144,7 +9154,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="19" spans="1:12">
+    <row r="19" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>617</v>
       </c>
@@ -9182,7 +9192,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="20" spans="1:12">
+    <row r="20" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>621</v>
       </c>
@@ -9220,7 +9230,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="21" spans="1:12">
+    <row r="21" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>626</v>
       </c>
@@ -9258,7 +9268,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="22" spans="1:12">
+    <row r="22" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>631</v>
       </c>
@@ -9296,7 +9306,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="23" spans="1:12">
+    <row r="23" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>635</v>
       </c>
@@ -9334,7 +9344,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="24" spans="1:12">
+    <row r="24" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>639</v>
       </c>
@@ -9372,7 +9382,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="25" spans="1:12">
+    <row r="25" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>643</v>
       </c>
@@ -9410,7 +9420,7 @@
         <v>612</v>
       </c>
     </row>
-    <row r="26" spans="1:12">
+    <row r="26" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>648</v>
       </c>
@@ -9448,7 +9458,7 @@
         <v>612</v>
       </c>
     </row>
-    <row r="27" spans="1:12">
+    <row r="27" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>653</v>
       </c>
@@ -9486,7 +9496,7 @@
         <v>612</v>
       </c>
     </row>
-    <row r="28" spans="1:12">
+    <row r="28" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>657</v>
       </c>
@@ -9524,7 +9534,7 @@
         <v>612</v>
       </c>
     </row>
-    <row r="29" spans="1:12">
+    <row r="29" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>661</v>
       </c>
@@ -9562,7 +9572,7 @@
         <v>612</v>
       </c>
     </row>
-    <row r="30" spans="1:12">
+    <row r="30" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>665</v>
       </c>
@@ -9600,7 +9610,7 @@
         <v>612</v>
       </c>
     </row>
-    <row r="31" spans="1:12">
+    <row r="31" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
         <v>670</v>
       </c>
@@ -9638,7 +9648,7 @@
         <v>612</v>
       </c>
     </row>
-    <row r="32" spans="1:12">
+    <row r="32" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
         <v>674</v>
       </c>
@@ -9676,7 +9686,7 @@
         <v>612</v>
       </c>
     </row>
-    <row r="33" spans="1:12">
+    <row r="33" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
         <v>678</v>
       </c>
@@ -9714,7 +9724,7 @@
         <v>612</v>
       </c>
     </row>
-    <row r="34" spans="1:12">
+    <row r="34" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
         <v>682</v>
       </c>
@@ -9752,7 +9762,7 @@
         <v>612</v>
       </c>
     </row>
-    <row r="35" spans="1:12">
+    <row r="35" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
         <v>686</v>
       </c>
@@ -9790,7 +9800,7 @@
         <v>612</v>
       </c>
     </row>
-    <row r="36" spans="1:12">
+    <row r="36" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
         <v>690</v>
       </c>
@@ -9828,7 +9838,7 @@
         <v>612</v>
       </c>
     </row>
-    <row r="37" spans="1:12">
+    <row r="37" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
         <v>694</v>
       </c>
@@ -9866,7 +9876,7 @@
         <v>612</v>
       </c>
     </row>
-    <row r="38" spans="1:12">
+    <row r="38" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
         <v>698</v>
       </c>
@@ -9904,7 +9914,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="39" spans="1:12">
+    <row r="39" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
         <v>704</v>
       </c>
@@ -9942,7 +9952,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="40" spans="1:12">
+    <row r="40" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
         <v>708</v>
       </c>
@@ -9980,7 +9990,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="41" spans="1:12">
+    <row r="41" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
         <v>713</v>
       </c>
@@ -10018,7 +10028,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="42" spans="1:12">
+    <row r="42" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
         <v>717</v>
       </c>
@@ -10056,7 +10066,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="43" spans="1:12">
+    <row r="43" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
         <v>721</v>
       </c>
@@ -10094,7 +10104,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="44" spans="1:12">
+    <row r="44" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
         <v>724</v>
       </c>
@@ -10132,7 +10142,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="45" spans="1:12">
+    <row r="45" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
         <v>731</v>
       </c>
@@ -10164,7 +10174,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="46" spans="1:12">
+    <row r="46" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
         <v>735</v>
       </c>
@@ -10196,7 +10206,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="47" spans="1:12">
+    <row r="47" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
         <v>739</v>
       </c>
@@ -10228,7 +10238,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="48" spans="1:12">
+    <row r="48" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
         <v>743</v>
       </c>
@@ -10260,7 +10270,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="49" spans="1:10">
+    <row r="49" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
         <v>747</v>
       </c>
@@ -10292,7 +10302,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="50" spans="1:10">
+    <row r="50" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
         <v>751</v>
       </c>
@@ -10324,7 +10334,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="51" spans="1:10">
+    <row r="51" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
         <v>755</v>
       </c>
@@ -10356,7 +10366,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="52" spans="1:10">
+    <row r="52" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
         <v>760</v>
       </c>
@@ -10388,7 +10398,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="53" spans="1:10">
+    <row r="53" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
         <v>764</v>
       </c>
@@ -10420,7 +10430,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="54" spans="1:10">
+    <row r="54" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
         <v>768</v>
       </c>
@@ -10452,7 +10462,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="55" spans="1:10">
+    <row r="55" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
         <v>772</v>
       </c>
@@ -10484,7 +10494,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="56" spans="1:10">
+    <row r="56" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
         <v>776</v>
       </c>
@@ -10516,7 +10526,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="57" spans="1:10">
+    <row r="57" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
         <v>780</v>
       </c>
@@ -10548,7 +10558,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="58" spans="1:10">
+    <row r="58" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
         <v>784</v>
       </c>
@@ -10580,7 +10590,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="59" spans="1:10">
+    <row r="59" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
         <v>788</v>
       </c>
@@ -10612,7 +10622,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="60" spans="1:10">
+    <row r="60" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
         <v>792</v>
       </c>
@@ -10644,7 +10654,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="61" spans="1:10">
+    <row r="61" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
         <v>796</v>
       </c>
@@ -10658,7 +10668,7 @@
         <v>70000</v>
       </c>
       <c r="E61">
-        <v>0.001</v>
+        <v>1E-3</v>
       </c>
       <c r="F61">
         <v>0</v>
@@ -10676,7 +10686,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="62" spans="1:10">
+    <row r="62" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
         <v>800</v>
       </c>
@@ -10690,7 +10700,7 @@
         <v>70000</v>
       </c>
       <c r="E62">
-        <v>0.001</v>
+        <v>1E-3</v>
       </c>
       <c r="F62">
         <v>0</v>
@@ -10708,7 +10718,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="63" spans="1:10">
+    <row r="63" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
         <v>804</v>
       </c>
@@ -10740,7 +10750,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="64" spans="1:10">
+    <row r="64" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
         <v>808</v>
       </c>
@@ -10772,7 +10782,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="65" spans="1:10">
+    <row r="65" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A65" t="s">
         <v>812</v>
       </c>
@@ -10804,7 +10814,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="66" spans="1:10">
+    <row r="66" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A66" t="s">
         <v>817</v>
       </c>
@@ -10836,7 +10846,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="67" spans="1:10">
+    <row r="67" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A67" t="s">
         <v>821</v>
       </c>
@@ -10868,7 +10878,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="68" spans="1:10">
+    <row r="68" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A68" t="s">
         <v>825</v>
       </c>
@@ -10900,7 +10910,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="69" spans="1:10">
+    <row r="69" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A69" t="s">
         <v>829</v>
       </c>
@@ -10932,7 +10942,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="70" spans="1:10">
+    <row r="70" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A70" t="s">
         <v>833</v>
       </c>
@@ -10964,7 +10974,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="71" spans="1:10">
+    <row r="71" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A71" t="s">
         <v>837</v>
       </c>
@@ -10996,7 +11006,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="72" spans="1:10">
+    <row r="72" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A72" t="s">
         <v>841</v>
       </c>
@@ -11034,11 +11044,11 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:Q183"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:17">
+    <row r="1" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>89</v>
       </c>
@@ -11067,7 +11077,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="2" spans="1:17">
+    <row r="2" spans="1:17" x14ac:dyDescent="0.2">
       <c r="D2" t="s">
         <v>533</v>
       </c>
@@ -11108,7 +11118,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="3" spans="1:17">
+    <row r="3" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>849</v>
       </c>
@@ -11149,7 +11159,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="4" spans="1:17">
+    <row r="4" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>853</v>
       </c>
@@ -11190,7 +11200,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="5" spans="1:17">
+    <row r="5" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>856</v>
       </c>
@@ -11231,7 +11241,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="6" spans="1:17">
+    <row r="6" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>859</v>
       </c>
@@ -11272,7 +11282,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="7" spans="1:17">
+    <row r="7" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>862</v>
       </c>
@@ -11313,7 +11323,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="8" spans="1:17">
+    <row r="8" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>865</v>
       </c>
@@ -11354,7 +11364,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="9" spans="1:17">
+    <row r="9" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>868</v>
       </c>
@@ -11395,7 +11405,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="10" spans="1:17">
+    <row r="10" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>871</v>
       </c>
@@ -11436,7 +11446,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="11" spans="1:17">
+    <row r="11" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>874</v>
       </c>
@@ -11477,7 +11487,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="12" spans="1:17">
+    <row r="12" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>877</v>
       </c>
@@ -11518,7 +11528,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="13" spans="1:17">
+    <row r="13" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>880</v>
       </c>
@@ -11559,7 +11569,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="14" spans="1:17">
+    <row r="14" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>884</v>
       </c>
@@ -11600,7 +11610,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="15" spans="1:17">
+    <row r="15" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>889</v>
       </c>
@@ -11638,7 +11648,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="16" spans="1:17">
+    <row r="16" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>893</v>
       </c>
@@ -11679,7 +11689,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="17" spans="1:14">
+    <row r="17" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>896</v>
       </c>
@@ -11720,7 +11730,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="18" spans="1:14">
+    <row r="18" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>899</v>
       </c>
@@ -11764,7 +11774,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="19" spans="1:14">
+    <row r="19" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>904</v>
       </c>
@@ -11808,7 +11818,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="20" spans="1:14">
+    <row r="20" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>908</v>
       </c>
@@ -11849,7 +11859,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="21" spans="1:14">
+    <row r="21" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>912</v>
       </c>
@@ -11890,7 +11900,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="22" spans="1:14">
+    <row r="22" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>915</v>
       </c>
@@ -11931,7 +11941,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="23" spans="1:14">
+    <row r="23" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>918</v>
       </c>
@@ -11972,7 +11982,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="24" spans="1:14">
+    <row r="24" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>571</v>
       </c>
@@ -11989,7 +11999,7 @@
         <v>70000</v>
       </c>
       <c r="F24">
-        <v>0.001</v>
+        <v>1E-3</v>
       </c>
       <c r="G24">
         <v>0</v>
@@ -12016,7 +12026,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="25" spans="1:14">
+    <row r="25" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>576</v>
       </c>
@@ -12033,7 +12043,7 @@
         <v>2147483647</v>
       </c>
       <c r="F25">
-        <v>0.001</v>
+        <v>1E-3</v>
       </c>
       <c r="G25">
         <v>0</v>
@@ -12060,7 +12070,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="26" spans="1:14">
+    <row r="26" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>581</v>
       </c>
@@ -12077,7 +12087,7 @@
         <v>0</v>
       </c>
       <c r="F26">
-        <v>0.001</v>
+        <v>1E-3</v>
       </c>
       <c r="G26">
         <v>0</v>
@@ -12104,7 +12114,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="27" spans="1:14">
+    <row r="27" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>585</v>
       </c>
@@ -12121,7 +12131,7 @@
         <v>2147483647</v>
       </c>
       <c r="F27">
-        <v>0.001</v>
+        <v>1E-3</v>
       </c>
       <c r="G27">
         <v>0</v>
@@ -12148,7 +12158,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="28" spans="1:14">
+    <row r="28" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>591</v>
       </c>
@@ -12192,7 +12202,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="29" spans="1:14">
+    <row r="29" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>595</v>
       </c>
@@ -12233,7 +12243,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="30" spans="1:14">
+    <row r="30" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>600</v>
       </c>
@@ -12277,7 +12287,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="31" spans="1:14">
+    <row r="31" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
         <v>605</v>
       </c>
@@ -12321,7 +12331,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="32" spans="1:14">
+    <row r="32" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
         <v>931</v>
       </c>
@@ -12365,7 +12375,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="33" spans="1:14">
+    <row r="33" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
         <v>935</v>
       </c>
@@ -12406,7 +12416,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="34" spans="1:14">
+    <row r="34" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
         <v>610</v>
       </c>
@@ -12450,7 +12460,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="35" spans="1:14">
+    <row r="35" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
         <v>625</v>
       </c>
@@ -12494,7 +12504,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="36" spans="1:14">
+    <row r="36" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
         <v>630</v>
       </c>
@@ -12538,7 +12548,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="37" spans="1:14">
+    <row r="37" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
         <v>646</v>
       </c>
@@ -12582,7 +12592,7 @@
         <v>612</v>
       </c>
     </row>
-    <row r="38" spans="1:14">
+    <row r="38" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
         <v>652</v>
       </c>
@@ -12626,7 +12636,7 @@
         <v>612</v>
       </c>
     </row>
-    <row r="39" spans="1:14">
+    <row r="39" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
         <v>656</v>
       </c>
@@ -12670,7 +12680,7 @@
         <v>612</v>
       </c>
     </row>
-    <row r="40" spans="1:14">
+    <row r="40" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
         <v>660</v>
       </c>
@@ -12714,7 +12724,7 @@
         <v>612</v>
       </c>
     </row>
-    <row r="41" spans="1:14">
+    <row r="41" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
         <v>664</v>
       </c>
@@ -12758,7 +12768,7 @@
         <v>612</v>
       </c>
     </row>
-    <row r="42" spans="1:14">
+    <row r="42" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
         <v>669</v>
       </c>
@@ -12802,7 +12812,7 @@
         <v>612</v>
       </c>
     </row>
-    <row r="43" spans="1:14">
+    <row r="43" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
         <v>673</v>
       </c>
@@ -12846,7 +12856,7 @@
         <v>612</v>
       </c>
     </row>
-    <row r="44" spans="1:14">
+    <row r="44" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
         <v>677</v>
       </c>
@@ -12890,7 +12900,7 @@
         <v>612</v>
       </c>
     </row>
-    <row r="45" spans="1:14">
+    <row r="45" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
         <v>681</v>
       </c>
@@ -12934,13 +12944,16 @@
         <v>612</v>
       </c>
     </row>
-    <row r="46" spans="1:14">
+    <row r="46" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
         <v>685</v>
       </c>
       <c r="B46" t="s">
         <v>683</v>
       </c>
+      <c r="C46">
+        <v>2</v>
+      </c>
       <c r="D46">
         <v>0</v>
       </c>
@@ -12975,7 +12988,7 @@
         <v>612</v>
       </c>
     </row>
-    <row r="47" spans="1:14">
+    <row r="47" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
         <v>689</v>
       </c>
@@ -13019,7 +13032,7 @@
         <v>612</v>
       </c>
     </row>
-    <row r="48" spans="1:14">
+    <row r="48" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
         <v>693</v>
       </c>
@@ -13063,7 +13076,7 @@
         <v>612</v>
       </c>
     </row>
-    <row r="49" spans="1:14">
+    <row r="49" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
         <v>697</v>
       </c>
@@ -13107,7 +13120,7 @@
         <v>612</v>
       </c>
     </row>
-    <row r="50" spans="1:14">
+    <row r="50" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
         <v>947</v>
       </c>
@@ -13148,7 +13161,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="51" spans="1:14">
+    <row r="51" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
         <v>950</v>
       </c>
@@ -13189,7 +13202,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="52" spans="1:14">
+    <row r="52" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
         <v>953</v>
       </c>
@@ -13230,7 +13243,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="53" spans="1:14">
+    <row r="53" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
         <v>956</v>
       </c>
@@ -13271,7 +13284,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="54" spans="1:14">
+    <row r="54" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
         <v>959</v>
       </c>
@@ -13312,7 +13325,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="55" spans="1:14">
+    <row r="55" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
         <v>963</v>
       </c>
@@ -13353,7 +13366,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="56" spans="1:14">
+    <row r="56" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
         <v>966</v>
       </c>
@@ -13394,7 +13407,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="57" spans="1:14">
+    <row r="57" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
         <v>969</v>
       </c>
@@ -13435,7 +13448,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="58" spans="1:14">
+    <row r="58" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
         <v>972</v>
       </c>
@@ -13476,7 +13489,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="59" spans="1:14">
+    <row r="59" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
         <v>975</v>
       </c>
@@ -13517,7 +13530,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="60" spans="1:14">
+    <row r="60" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
         <v>978</v>
       </c>
@@ -13558,7 +13571,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="61" spans="1:14">
+    <row r="61" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
         <v>981</v>
       </c>
@@ -13599,7 +13612,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="62" spans="1:14">
+    <row r="62" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
         <v>984</v>
       </c>
@@ -13640,7 +13653,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="63" spans="1:14">
+    <row r="63" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
         <v>702</v>
       </c>
@@ -13684,7 +13697,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="64" spans="1:14">
+    <row r="64" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
         <v>707</v>
       </c>
@@ -13728,7 +13741,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="65" spans="1:14">
+    <row r="65" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A65" t="s">
         <v>712</v>
       </c>
@@ -13772,7 +13785,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="66" spans="1:14">
+    <row r="66" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A66" t="s">
         <v>716</v>
       </c>
@@ -13816,7 +13829,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="67" spans="1:14">
+    <row r="67" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A67" t="s">
         <v>719</v>
       </c>
@@ -13860,7 +13873,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="68" spans="1:14">
+    <row r="68" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A68" t="s">
         <v>723</v>
       </c>
@@ -13904,7 +13917,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="69" spans="1:14">
+    <row r="69" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A69" t="s">
         <v>728</v>
       </c>
@@ -13948,7 +13961,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="70" spans="1:14">
+    <row r="70" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A70" t="s">
         <v>989</v>
       </c>
@@ -13983,7 +13996,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="71" spans="1:14">
+    <row r="71" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A71" t="s">
         <v>992</v>
       </c>
@@ -14018,7 +14031,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="72" spans="1:14">
+    <row r="72" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A72" t="s">
         <v>995</v>
       </c>
@@ -14053,7 +14066,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="73" spans="1:14">
+    <row r="73" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A73" t="s">
         <v>998</v>
       </c>
@@ -14088,7 +14101,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="74" spans="1:14">
+    <row r="74" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A74" t="s">
         <v>1001</v>
       </c>
@@ -14105,7 +14118,7 @@
         <v>70000</v>
       </c>
       <c r="F74">
-        <v>0.001</v>
+        <v>1E-3</v>
       </c>
       <c r="G74">
         <v>0</v>
@@ -14123,7 +14136,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="75" spans="1:14">
+    <row r="75" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A75" t="s">
         <v>1004</v>
       </c>
@@ -14158,7 +14171,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="76" spans="1:14">
+    <row r="76" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A76" t="s">
         <v>1007</v>
       </c>
@@ -14193,7 +14206,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="77" spans="1:14">
+    <row r="77" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A77" t="s">
         <v>1010</v>
       </c>
@@ -14228,7 +14241,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="78" spans="1:14">
+    <row r="78" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A78" t="s">
         <v>1013</v>
       </c>
@@ -14263,7 +14276,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="79" spans="1:14">
+    <row r="79" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A79" t="s">
         <v>1016</v>
       </c>
@@ -14298,7 +14311,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="80" spans="1:14">
+    <row r="80" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A80" t="s">
         <v>1019</v>
       </c>
@@ -14333,7 +14346,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="81" spans="1:12">
+    <row r="81" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A81" t="s">
         <v>1022</v>
       </c>
@@ -14368,7 +14381,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="82" spans="1:12">
+    <row r="82" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A82" t="s">
         <v>1025</v>
       </c>
@@ -14403,7 +14416,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="83" spans="1:12">
+    <row r="83" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A83" t="s">
         <v>1028</v>
       </c>
@@ -14438,7 +14451,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="84" spans="1:12">
+    <row r="84" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A84" t="s">
         <v>1031</v>
       </c>
@@ -14473,7 +14486,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="85" spans="1:12">
+    <row r="85" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A85" t="s">
         <v>1035</v>
       </c>
@@ -14508,7 +14521,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="86" spans="1:12">
+    <row r="86" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A86" t="s">
         <v>1038</v>
       </c>
@@ -14543,7 +14556,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="87" spans="1:12">
+    <row r="87" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A87" t="s">
         <v>1041</v>
       </c>
@@ -14578,7 +14591,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="88" spans="1:12">
+    <row r="88" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A88" t="s">
         <v>1044</v>
       </c>
@@ -14613,7 +14626,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="89" spans="1:12">
+    <row r="89" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A89" t="s">
         <v>1047</v>
       </c>
@@ -14648,7 +14661,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="90" spans="1:12">
+    <row r="90" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A90" t="s">
         <v>1050</v>
       </c>
@@ -14683,7 +14696,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="91" spans="1:12">
+    <row r="91" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A91" t="s">
         <v>1053</v>
       </c>
@@ -14718,7 +14731,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="92" spans="1:12">
+    <row r="92" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A92" t="s">
         <v>1056</v>
       </c>
@@ -14753,7 +14766,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="93" spans="1:12">
+    <row r="93" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A93" t="s">
         <v>1059</v>
       </c>
@@ -14788,7 +14801,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="94" spans="1:12">
+    <row r="94" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A94" t="s">
         <v>1062</v>
       </c>
@@ -14823,7 +14836,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="95" spans="1:12">
+    <row r="95" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A95" t="s">
         <v>734</v>
       </c>
@@ -14861,7 +14874,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="96" spans="1:12">
+    <row r="96" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A96" t="s">
         <v>738</v>
       </c>
@@ -14899,7 +14912,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="97" spans="1:12">
+    <row r="97" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A97" t="s">
         <v>742</v>
       </c>
@@ -14937,7 +14950,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="98" spans="1:12">
+    <row r="98" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A98" t="s">
         <v>746</v>
       </c>
@@ -14975,7 +14988,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="99" spans="1:12">
+    <row r="99" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A99" t="s">
         <v>750</v>
       </c>
@@ -15013,7 +15026,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="100" spans="1:12">
+    <row r="100" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A100" t="s">
         <v>754</v>
       </c>
@@ -15051,7 +15064,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="101" spans="1:12">
+    <row r="101" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A101" t="s">
         <v>759</v>
       </c>
@@ -15089,7 +15102,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="102" spans="1:12">
+    <row r="102" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A102" t="s">
         <v>763</v>
       </c>
@@ -15127,7 +15140,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="103" spans="1:12">
+    <row r="103" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A103" t="s">
         <v>767</v>
       </c>
@@ -15165,7 +15178,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="104" spans="1:12">
+    <row r="104" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A104" t="s">
         <v>771</v>
       </c>
@@ -15203,7 +15216,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="105" spans="1:12">
+    <row r="105" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A105" t="s">
         <v>775</v>
       </c>
@@ -15241,7 +15254,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="106" spans="1:12">
+    <row r="106" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A106" t="s">
         <v>779</v>
       </c>
@@ -15279,7 +15292,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="107" spans="1:12">
+    <row r="107" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A107" t="s">
         <v>1071</v>
       </c>
@@ -15314,7 +15327,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="108" spans="1:12">
+    <row r="108" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A108" t="s">
         <v>1074</v>
       </c>
@@ -15349,7 +15362,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="109" spans="1:12">
+    <row r="109" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A109" t="s">
         <v>1077</v>
       </c>
@@ -15384,7 +15397,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="110" spans="1:12">
+    <row r="110" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A110" t="s">
         <v>1080</v>
       </c>
@@ -15419,7 +15432,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="111" spans="1:12">
+    <row r="111" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A111" t="s">
         <v>1083</v>
       </c>
@@ -15454,7 +15467,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="112" spans="1:12">
+    <row r="112" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A112" t="s">
         <v>1086</v>
       </c>
@@ -15489,7 +15502,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="113" spans="1:12">
+    <row r="113" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A113" t="s">
         <v>1089</v>
       </c>
@@ -15524,7 +15537,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="114" spans="1:12">
+    <row r="114" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A114" t="s">
         <v>1092</v>
       </c>
@@ -15559,7 +15572,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="115" spans="1:12">
+    <row r="115" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A115" t="s">
         <v>1096</v>
       </c>
@@ -15594,7 +15607,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="116" spans="1:12">
+    <row r="116" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A116" t="s">
         <v>1100</v>
       </c>
@@ -15629,7 +15642,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="117" spans="1:12">
+    <row r="117" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A117" t="s">
         <v>1103</v>
       </c>
@@ -15664,7 +15677,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="118" spans="1:12">
+    <row r="118" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A118" t="s">
         <v>1106</v>
       </c>
@@ -15699,7 +15712,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="119" spans="1:12">
+    <row r="119" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A119" t="s">
         <v>1109</v>
       </c>
@@ -15734,7 +15747,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="120" spans="1:12">
+    <row r="120" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A120" t="s">
         <v>1112</v>
       </c>
@@ -15769,7 +15782,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="121" spans="1:12">
+    <row r="121" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A121" t="s">
         <v>1115</v>
       </c>
@@ -15804,7 +15817,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="122" spans="1:12">
+    <row r="122" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A122" t="s">
         <v>1118</v>
       </c>
@@ -15839,7 +15852,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="123" spans="1:12">
+    <row r="123" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A123" t="s">
         <v>1121</v>
       </c>
@@ -15874,7 +15887,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="124" spans="1:12">
+    <row r="124" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A124" t="s">
         <v>1124</v>
       </c>
@@ -15909,7 +15922,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="125" spans="1:12">
+    <row r="125" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A125" t="s">
         <v>1127</v>
       </c>
@@ -15944,7 +15957,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="126" spans="1:12">
+    <row r="126" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A126" t="s">
         <v>1130</v>
       </c>
@@ -15979,7 +15992,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="127" spans="1:12">
+    <row r="127" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A127" t="s">
         <v>1133</v>
       </c>
@@ -16014,7 +16027,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="128" spans="1:12">
+    <row r="128" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A128" t="s">
         <v>1136</v>
       </c>
@@ -16049,7 +16062,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="129" spans="1:12">
+    <row r="129" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A129" t="s">
         <v>1139</v>
       </c>
@@ -16084,7 +16097,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="130" spans="1:12">
+    <row r="130" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A130" t="s">
         <v>1142</v>
       </c>
@@ -16119,7 +16132,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="131" spans="1:12">
+    <row r="131" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A131" t="s">
         <v>1145</v>
       </c>
@@ -16154,7 +16167,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="132" spans="1:12">
+    <row r="132" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A132" t="s">
         <v>1148</v>
       </c>
@@ -16189,7 +16202,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="133" spans="1:12">
+    <row r="133" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A133" t="s">
         <v>1151</v>
       </c>
@@ -16224,7 +16237,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="134" spans="1:12">
+    <row r="134" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A134" t="s">
         <v>1154</v>
       </c>
@@ -16259,7 +16272,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="135" spans="1:12">
+    <row r="135" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A135" t="s">
         <v>1157</v>
       </c>
@@ -16294,7 +16307,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="136" spans="1:12">
+    <row r="136" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A136" t="s">
         <v>1160</v>
       </c>
@@ -16329,7 +16342,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="137" spans="1:12">
+    <row r="137" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A137" t="s">
         <v>1163</v>
       </c>
@@ -16364,7 +16377,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="138" spans="1:12">
+    <row r="138" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A138" t="s">
         <v>1166</v>
       </c>
@@ -16399,7 +16412,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="139" spans="1:12">
+    <row r="139" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A139" t="s">
         <v>1169</v>
       </c>
@@ -16434,7 +16447,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="140" spans="1:12">
+    <row r="140" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A140" t="s">
         <v>1172</v>
       </c>
@@ -16469,7 +16482,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="141" spans="1:12">
+    <row r="141" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A141" t="s">
         <v>1176</v>
       </c>
@@ -16504,7 +16517,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="142" spans="1:12">
+    <row r="142" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A142" t="s">
         <v>1179</v>
       </c>
@@ -16539,7 +16552,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="143" spans="1:12">
+    <row r="143" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A143" t="s">
         <v>783</v>
       </c>
@@ -16577,7 +16590,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="144" spans="1:12">
+    <row r="144" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A144" t="s">
         <v>787</v>
       </c>
@@ -16615,7 +16628,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="145" spans="1:12">
+    <row r="145" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A145" t="s">
         <v>791</v>
       </c>
@@ -16653,7 +16666,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="146" spans="1:12">
+    <row r="146" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A146" t="s">
         <v>795</v>
       </c>
@@ -16691,7 +16704,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="147" spans="1:12">
+    <row r="147" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A147" t="s">
         <v>799</v>
       </c>
@@ -16729,7 +16742,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="148" spans="1:12">
+    <row r="148" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A148" t="s">
         <v>803</v>
       </c>
@@ -16767,7 +16780,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="149" spans="1:12">
+    <row r="149" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A149" t="s">
         <v>807</v>
       </c>
@@ -16805,7 +16818,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="150" spans="1:12">
+    <row r="150" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A150" t="s">
         <v>811</v>
       </c>
@@ -16843,7 +16856,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="151" spans="1:12">
+    <row r="151" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A151" t="s">
         <v>816</v>
       </c>
@@ -16881,7 +16894,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="152" spans="1:12">
+    <row r="152" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A152" t="s">
         <v>820</v>
       </c>
@@ -16919,7 +16932,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="153" spans="1:12">
+    <row r="153" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A153" t="s">
         <v>824</v>
       </c>
@@ -16957,7 +16970,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="154" spans="1:12">
+    <row r="154" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A154" t="s">
         <v>828</v>
       </c>
@@ -16995,7 +17008,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="155" spans="1:12">
+    <row r="155" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A155" t="s">
         <v>1186</v>
       </c>
@@ -17030,7 +17043,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="156" spans="1:12">
+    <row r="156" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A156" t="s">
         <v>1189</v>
       </c>
@@ -17065,7 +17078,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="157" spans="1:12">
+    <row r="157" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A157" t="s">
         <v>1192</v>
       </c>
@@ -17100,7 +17113,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="158" spans="1:12">
+    <row r="158" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A158" t="s">
         <v>1196</v>
       </c>
@@ -17135,7 +17148,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="159" spans="1:12">
+    <row r="159" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A159" t="s">
         <v>1199</v>
       </c>
@@ -17170,7 +17183,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="160" spans="1:12">
+    <row r="160" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A160" t="s">
         <v>1202</v>
       </c>
@@ -17205,7 +17218,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="161" spans="1:12">
+    <row r="161" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A161" t="s">
         <v>1205</v>
       </c>
@@ -17240,7 +17253,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="162" spans="1:12">
+    <row r="162" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A162" t="s">
         <v>1208</v>
       </c>
@@ -17275,7 +17288,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="163" spans="1:12">
+    <row r="163" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A163" t="s">
         <v>1211</v>
       </c>
@@ -17310,7 +17323,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="164" spans="1:12">
+    <row r="164" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A164" t="s">
         <v>1214</v>
       </c>
@@ -17345,7 +17358,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="165" spans="1:12">
+    <row r="165" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A165" t="s">
         <v>1217</v>
       </c>
@@ -17380,7 +17393,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="166" spans="1:12">
+    <row r="166" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A166" t="s">
         <v>1220</v>
       </c>
@@ -17415,7 +17428,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="167" spans="1:12">
+    <row r="167" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A167" t="s">
         <v>1223</v>
       </c>
@@ -17450,7 +17463,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="168" spans="1:12">
+    <row r="168" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A168" t="s">
         <v>1226</v>
       </c>
@@ -17467,7 +17480,7 @@
         <v>2147483647</v>
       </c>
       <c r="F168">
-        <v>0.001</v>
+        <v>1E-3</v>
       </c>
       <c r="G168">
         <v>0</v>
@@ -17485,7 +17498,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="169" spans="1:12">
+    <row r="169" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A169" t="s">
         <v>1229</v>
       </c>
@@ -17502,7 +17515,7 @@
         <v>2147483647</v>
       </c>
       <c r="F169">
-        <v>0.001</v>
+        <v>1E-3</v>
       </c>
       <c r="G169">
         <v>0</v>
@@ -17520,7 +17533,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="170" spans="1:12">
+    <row r="170" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A170" t="s">
         <v>1232</v>
       </c>
@@ -17555,7 +17568,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="171" spans="1:12">
+    <row r="171" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A171" t="s">
         <v>1235</v>
       </c>
@@ -17590,7 +17603,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="172" spans="1:12">
+    <row r="172" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A172" t="s">
         <v>1238</v>
       </c>
@@ -17625,7 +17638,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="173" spans="1:12">
+    <row r="173" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A173" t="s">
         <v>1241</v>
       </c>
@@ -17660,7 +17673,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="174" spans="1:12">
+    <row r="174" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A174" t="s">
         <v>1244</v>
       </c>
@@ -17695,7 +17708,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="175" spans="1:12">
+    <row r="175" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A175" t="s">
         <v>1247</v>
       </c>
@@ -17730,7 +17743,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="176" spans="1:12">
+    <row r="176" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A176" t="s">
         <v>1250</v>
       </c>
@@ -17765,7 +17778,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="177" spans="1:12">
+    <row r="177" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A177" t="s">
         <v>1253</v>
       </c>
@@ -17800,7 +17813,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="178" spans="1:12">
+    <row r="178" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A178" t="s">
         <v>1256</v>
       </c>
@@ -17835,7 +17848,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="179" spans="1:12">
+    <row r="179" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A179" t="s">
         <v>832</v>
       </c>
@@ -17873,7 +17886,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="180" spans="1:12">
+    <row r="180" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A180" t="s">
         <v>836</v>
       </c>
@@ -17911,7 +17924,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="181" spans="1:12">
+    <row r="181" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A181" t="s">
         <v>840</v>
       </c>
@@ -17949,7 +17962,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="182" spans="1:12">
+    <row r="182" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A182" t="s">
         <v>844</v>
       </c>
@@ -17987,7 +18000,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="183" spans="1:12">
+    <row r="183" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A183" t="s">
         <v>1262</v>
       </c>
@@ -18028,11 +18041,11 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:J6"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:10">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>89</v>
       </c>
@@ -18058,7 +18071,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="2" spans="1:10">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
       <c r="F2" t="s">
         <v>96</v>
       </c>
@@ -18075,7 +18088,7 @@
         <v>538</v>
       </c>
     </row>
-    <row r="3" spans="1:10">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>1269</v>
       </c>
@@ -18098,7 +18111,7 @@
         <v>1273</v>
       </c>
     </row>
-    <row r="4" spans="1:10">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>1274</v>
       </c>
@@ -18121,7 +18134,7 @@
         <v>1273</v>
       </c>
     </row>
-    <row r="5" spans="1:10">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>1277</v>
       </c>
@@ -18144,7 +18157,7 @@
         <v>1273</v>
       </c>
     </row>
-    <row r="6" spans="1:10">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>1280</v>
       </c>
@@ -18173,11 +18186,11 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:1">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>1283</v>
       </c>

</xml_diff>

<commit_message>
Modify profiles to match the published CDPT
</commit_message>
<xml_diff>
--- a/data/profiles/mandatory_1547.xlsx
+++ b/data/profiles/mandatory_1547.xlsx
@@ -6326,11 +6326,15 @@
       <c r="C34">
         <v>1</v>
       </c>
-      <c r="D34" t="s">
-        <v>243</v>
-      </c>
-      <c r="E34" t="s">
-        <v>244</v>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Normal: No Active Communications Error </t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Alarm: Active Communications Error </t>
+        </is>
       </c>
       <c r="F34" t="s">
         <v>245</v>
@@ -9390,10 +9394,10 @@
         <v>644</v>
       </c>
       <c r="C25">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D25">
-        <v>100</v>
+        <v>2147483647</v>
       </c>
       <c r="E25">
         <v>1</v>
@@ -9431,7 +9435,7 @@
         <v>0</v>
       </c>
       <c r="D26">
-        <v>100</v>
+        <v>20</v>
       </c>
       <c r="E26">
         <v>1</v>
@@ -9507,7 +9511,7 @@
         <v>0</v>
       </c>
       <c r="D28">
-        <v>100</v>
+        <v>255</v>
       </c>
       <c r="E28">
         <v>1</v>
@@ -9545,7 +9549,7 @@
         <v>0</v>
       </c>
       <c r="D29">
-        <v>100</v>
+        <v>255</v>
       </c>
       <c r="E29">
         <v>1</v>
@@ -9887,10 +9891,10 @@
         <v>0</v>
       </c>
       <c r="D38">
-        <v>100</v>
+        <v>2147483647</v>
       </c>
       <c r="E38">
-        <v>1</v>
+        <v>0.001</v>
       </c>
       <c r="F38">
         <v>0</v>
@@ -9925,10 +9929,10 @@
         <v>0</v>
       </c>
       <c r="D39">
-        <v>100</v>
+        <v>2147483647</v>
       </c>
       <c r="E39">
-        <v>1</v>
+        <v>0.001</v>
       </c>
       <c r="F39">
         <v>0</v>
@@ -9963,10 +9967,10 @@
         <v>0</v>
       </c>
       <c r="D40">
-        <v>100</v>
+        <v>2147483647</v>
       </c>
       <c r="E40">
-        <v>1</v>
+        <v>0.001</v>
       </c>
       <c r="F40">
         <v>0</v>
@@ -10001,10 +10005,10 @@
         <v>0</v>
       </c>
       <c r="D41">
-        <v>100</v>
+        <v>2147483647</v>
       </c>
       <c r="E41">
-        <v>1</v>
+        <v>0.001</v>
       </c>
       <c r="F41">
         <v>0</v>
@@ -10036,10 +10040,10 @@
         <v>597</v>
       </c>
       <c r="C42">
-        <v>0</v>
+        <v>-2147483648</v>
       </c>
       <c r="D42">
-        <v>100</v>
+        <v>2147483647</v>
       </c>
       <c r="E42">
         <v>1</v>
@@ -10074,10 +10078,10 @@
         <v>603</v>
       </c>
       <c r="C43">
-        <v>0</v>
+        <v>-2147483648</v>
       </c>
       <c r="D43">
-        <v>100</v>
+        <v>2147483647</v>
       </c>
       <c r="E43">
         <v>1</v>
@@ -10112,10 +10116,10 @@
         <v>725</v>
       </c>
       <c r="C44">
-        <v>0</v>
+        <v>-2147483648</v>
       </c>
       <c r="D44">
-        <v>100</v>
+        <v>2147483647</v>
       </c>
       <c r="E44">
         <v>1</v>
@@ -12559,10 +12563,10 @@
         <v>2</v>
       </c>
       <c r="D37">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E37">
-        <v>100</v>
+        <v>2147483647</v>
       </c>
       <c r="F37">
         <v>1</v>
@@ -12577,7 +12581,7 @@
         <v>645</v>
       </c>
       <c r="J37">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K37" t="s">
         <v>643</v>
@@ -12606,7 +12610,7 @@
         <v>0</v>
       </c>
       <c r="E38">
-        <v>100</v>
+        <v>20</v>
       </c>
       <c r="F38">
         <v>1</v>
@@ -12694,7 +12698,7 @@
         <v>0</v>
       </c>
       <c r="E40">
-        <v>100</v>
+        <v>255</v>
       </c>
       <c r="F40">
         <v>1</v>
@@ -12738,7 +12742,7 @@
         <v>0</v>
       </c>
       <c r="E41">
-        <v>100</v>
+        <v>255</v>
       </c>
       <c r="F41">
         <v>1</v>
@@ -13134,10 +13138,10 @@
         <v>0</v>
       </c>
       <c r="E50">
-        <v>100</v>
+        <v>70000</v>
       </c>
       <c r="F50">
-        <v>1</v>
+        <v>0.001</v>
       </c>
       <c r="G50">
         <v>0</v>
@@ -13172,10 +13176,10 @@
         <v>3</v>
       </c>
       <c r="D51">
-        <v>0</v>
+        <v>-2147483648</v>
       </c>
       <c r="E51">
-        <v>100</v>
+        <v>2147483647</v>
       </c>
       <c r="F51">
         <v>1</v>
@@ -13213,10 +13217,10 @@
         <v>3</v>
       </c>
       <c r="D52">
-        <v>0</v>
+        <v>-2147483648</v>
       </c>
       <c r="E52">
-        <v>100</v>
+        <v>2147483647</v>
       </c>
       <c r="F52">
         <v>1</v>
@@ -13257,10 +13261,10 @@
         <v>0</v>
       </c>
       <c r="E53">
-        <v>100</v>
+        <v>2147483647</v>
       </c>
       <c r="F53">
-        <v>1</v>
+        <v>0.1</v>
       </c>
       <c r="G53">
         <v>0</v>
@@ -13298,10 +13302,10 @@
         <v>0</v>
       </c>
       <c r="E54">
-        <v>100</v>
+        <v>3600</v>
       </c>
       <c r="F54">
-        <v>1</v>
+        <v>0.1</v>
       </c>
       <c r="G54">
         <v>0</v>
@@ -13339,10 +13343,10 @@
         <v>0</v>
       </c>
       <c r="E55">
-        <v>100</v>
+        <v>2147483647</v>
       </c>
       <c r="F55">
-        <v>1</v>
+        <v>0.1</v>
       </c>
       <c r="G55">
         <v>0</v>
@@ -13380,10 +13384,10 @@
         <v>0</v>
       </c>
       <c r="E56">
-        <v>100</v>
+        <v>3600</v>
       </c>
       <c r="F56">
-        <v>1</v>
+        <v>0.1</v>
       </c>
       <c r="G56">
         <v>0</v>
@@ -13421,10 +13425,10 @@
         <v>0</v>
       </c>
       <c r="E57">
-        <v>100</v>
+        <v>2147483647</v>
       </c>
       <c r="F57">
-        <v>1</v>
+        <v>0.1</v>
       </c>
       <c r="G57">
         <v>0</v>
@@ -13462,10 +13466,10 @@
         <v>0</v>
       </c>
       <c r="E58">
-        <v>100</v>
+        <v>3600</v>
       </c>
       <c r="F58">
-        <v>1</v>
+        <v>0.1</v>
       </c>
       <c r="G58">
         <v>0</v>
@@ -13503,10 +13507,10 @@
         <v>0</v>
       </c>
       <c r="E59">
-        <v>100</v>
+        <v>2147483647</v>
       </c>
       <c r="F59">
-        <v>1</v>
+        <v>0.1</v>
       </c>
       <c r="G59">
         <v>0</v>
@@ -13541,13 +13545,13 @@
         <v>1</v>
       </c>
       <c r="D60">
-        <v>0</v>
+        <v>-2147483648</v>
       </c>
       <c r="E60">
-        <v>100</v>
+        <v>2147483647</v>
       </c>
       <c r="F60">
-        <v>1</v>
+        <v>0.1</v>
       </c>
       <c r="G60">
         <v>0</v>
@@ -13582,13 +13586,13 @@
         <v>1</v>
       </c>
       <c r="D61">
-        <v>0</v>
+        <v>-2147483648</v>
       </c>
       <c r="E61">
-        <v>100</v>
+        <v>2147483647</v>
       </c>
       <c r="F61">
-        <v>1</v>
+        <v>0.1</v>
       </c>
       <c r="G61">
         <v>0</v>
@@ -13623,13 +13627,13 @@
         <v>1</v>
       </c>
       <c r="D62">
-        <v>0</v>
+        <v>-2147483648</v>
       </c>
       <c r="E62">
-        <v>100</v>
+        <v>2147483647</v>
       </c>
       <c r="F62">
-        <v>1</v>
+        <v>0.1</v>
       </c>
       <c r="G62">
         <v>0</v>
@@ -13667,10 +13671,10 @@
         <v>0</v>
       </c>
       <c r="E63">
-        <v>100</v>
+        <v>2147483647</v>
       </c>
       <c r="F63">
-        <v>1</v>
+        <v>0.001</v>
       </c>
       <c r="G63">
         <v>0</v>
@@ -13711,10 +13715,10 @@
         <v>0</v>
       </c>
       <c r="E64">
-        <v>100</v>
+        <v>2147483647</v>
       </c>
       <c r="F64">
-        <v>1</v>
+        <v>0.001</v>
       </c>
       <c r="G64">
         <v>0</v>
@@ -13755,10 +13759,10 @@
         <v>0</v>
       </c>
       <c r="E65">
-        <v>100</v>
+        <v>2147483647</v>
       </c>
       <c r="F65">
-        <v>1</v>
+        <v>0.001</v>
       </c>
       <c r="G65">
         <v>0</v>
@@ -13799,10 +13803,10 @@
         <v>0</v>
       </c>
       <c r="E66">
-        <v>100</v>
+        <v>2147483647</v>
       </c>
       <c r="F66">
-        <v>1</v>
+        <v>0.001</v>
       </c>
       <c r="G66">
         <v>0</v>
@@ -13840,10 +13844,10 @@
         <v>2</v>
       </c>
       <c r="D67">
-        <v>0</v>
+        <v>-2147483648</v>
       </c>
       <c r="E67">
-        <v>100</v>
+        <v>2147483647</v>
       </c>
       <c r="F67">
         <v>1</v>
@@ -13884,10 +13888,10 @@
         <v>2</v>
       </c>
       <c r="D68">
-        <v>0</v>
+        <v>-2147483648</v>
       </c>
       <c r="E68">
-        <v>100</v>
+        <v>2147483647</v>
       </c>
       <c r="F68">
         <v>1</v>
@@ -13928,10 +13932,10 @@
         <v>2</v>
       </c>
       <c r="D69">
-        <v>0</v>
+        <v>-2147483648</v>
       </c>
       <c r="E69">
-        <v>100</v>
+        <v>2147483647</v>
       </c>
       <c r="F69">
         <v>1</v>

</xml_diff>